<commit_message>
chore: remove Gemini API code, simplify to native Apple Vision ML and Tesseract OCR
</commit_message>
<xml_diff>
--- a/backend/data/business_cards.xlsx
+++ b/backend/data/business_cards.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Business Cards" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business Cards'!$A$1:$K$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business Cards'!$A$1:$K$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -151,14 +151,14 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -601,7 +601,7 @@
     <row r="2" ht="120" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>40556bbf</t>
+          <t>8f0ca39c</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -642,7 +642,7 @@
       <c r="I2" s="7" t="inlineStr"/>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:08:36</t>
+          <t>2026-10-27 18:01:48</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
@@ -663,43 +663,105 @@
     <row r="3" ht="120" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
+          <t>40556bbf</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Alexander Wright</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>CHIEF EXECUTIVE OFFICER</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Nova Dynamics Inc.</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>+1 (415) 890-2341</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>alex@novadynamics.io</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>www.novadynamics.io</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>500 Howard St, Suite 400, San Francisco, CA 94105</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr"/>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:08:36</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>N
+Nova Dynamics Inc.
+Alexander Wright
+CHIEF EXECUTIVE OFFICER
+Phone: +1 (415) 890-2341
+Office Address:
+Email: alex@novadynamics.io
+500 Howard St, Suite 400
+Web: www.novadynamics.io
+San Francisco, CA 94105</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>b9569968</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>GOLD • SILVER • DIAMOND</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr"/>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>SS JEWELLERS</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>7016622431, 7862822743</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr"/>
-      <c r="G3" s="10" t="inlineStr"/>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>G-5. KUBER PLAZA, TEEN RASTA CIRCLE, ANKLESHWAR-393001.</t>
         </is>
       </c>
-      <c r="I3" s="12" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>SUNIL SONI | SAGAR SONI</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>2026-10-27 17:01:32</t>
         </is>
       </c>
-      <c r="K3" s="12" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>SUNIL SONI
 SAGAR SONI
@@ -712,38 +774,38 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="108" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="108" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>adea6ad3</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr"/>
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Krishna jewellers</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>9825 395021</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="inlineStr"/>
+      <c r="H5" s="13" t="inlineStr">
         <is>
           <t>Dukaan number 1 Mulla Wada Ankleshwar</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr"/>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr"/>
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:45:08</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>DOL
 Isall 9.
@@ -754,50 +816,50 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="108" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="6" ht="108" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>0f9731bd</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>markandeshwarofficial</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr"/>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Markandeshwar jewellers </t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>+91 757 582 6665</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>ommarkandeshwarjewellers@gmail.com</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr"/>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Shop No. A-6-7, Ganesh Plaza, Ground Floor, 500 Qtrs. Road</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>G.I.D.C., Ankleshwar - 393 002</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:44:13</t>
         </is>
       </c>
-      <c r="K5" s="12" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>Shop No. A-6-7, Ganesh Plaza,
 M: +91 757 582 6665
@@ -808,46 +870,46 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="120" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7" ht="120" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>b4746239</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>BHAVESH SON</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr"/>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Madhuram jewellers </t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>+91 90330 50916, +9194278 7937</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Shopping Center, Opp. Tr, Rasta Circle, Station Road</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>MADHURAM | JEWELLERS | Ankleshwar - 393 001</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J7" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:43:35</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="K7" s="13" t="inlineStr">
         <is>
           <t>L +9194278 7937）
 &amp; BHAVESH SON
@@ -861,46 +923,46 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="120" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="8" ht="120" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>6493cb67</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>GOLD • SILVER + DIAMOND</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>SS JEWELLERS</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>7016622431, 7862822743</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="10" t="inlineStr"/>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>G-5, KUBER PLAZA, TEEN RASTA CIRCLE, ANKLESHWAR-393001.</t>
         </is>
       </c>
-      <c r="I7" s="12" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>SUNIL SONI | SAGAR SONI</t>
         </is>
       </c>
-      <c r="J7" s="13" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:43:08</t>
         </is>
       </c>
-      <c r="K7" s="12" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>SUNIL SONI
 SAGAR SONI
@@ -913,38 +975,38 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="120" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9" ht="120" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>269f5a89</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr"/>
+      <c r="C9" s="10" t="inlineStr"/>
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Ruchit jewellers </t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>84607 84916, 85116 52185</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr"/>
+      <c r="G9" s="10" t="inlineStr"/>
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>Juna shakha market Nisha mein jaani restaurant nibaj Chhota bajar Ankleshwar</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="I9" s="13" t="inlineStr"/>
+      <c r="J9" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:41:31</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="K9" s="13" t="inlineStr">
         <is>
           <t>Med ข้อ
 鸟
@@ -969,38 +1031,38 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="120" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10" ht="120" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>9833f875</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Shree dagina jewellers </t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>90543 15911, 70436 15911</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr"/>
-      <c r="G9" s="10" t="inlineStr"/>
-      <c r="H9" s="12" t="inlineStr"/>
-      <c r="I9" s="12" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  Ganesh mithai Nisha mein Chhota Baja ankaleshwar,Vibrant mole,Mota Mandir road,kosamba, Surat</t>
         </is>
       </c>
-      <c r="J9" s="13" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:39:40</t>
         </is>
       </c>
-      <c r="K9" s="12" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>^ed aicl
 eiscaaz : 90543 15911
@@ -1014,58 +1076,58 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="120" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11" ht="120" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>2ba1b687</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Marcus Chen</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>PRINCIPAL ARCHITECT</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>Kroma Design Studio LLC</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>+1 (312) 880-9942</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>marcus@kromadesign.com</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>www.kromadesign.com</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>1200 N Michigan Ave, Chicago</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I11" s="13" t="inlineStr">
         <is>
           <t>IL 60611</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="J11" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:37:42</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="K11" s="13" t="inlineStr">
         <is>
           <t>K
 Kroma Design Studio LLC
@@ -1080,58 +1142,58 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="120" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>730479bf</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Dr. Elena Rostova, MD</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>A Aura Health Partners LLC</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>CHIEF CARDIOLOGIST &amp; PARTNER</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>+1 (212) 555-0198</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>e.rostova@aurahealth.com</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>aurahealth.com</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>742 Park Avenue, New York</t>
         </is>
       </c>
-      <c r="I11" s="12" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>NY 10021</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:37:41</t>
         </is>
       </c>
-      <c r="K11" s="12" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>A Aura Health Partners LLC
 Dr. Elena Rostova, MD
@@ -1145,54 +1207,54 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="120" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>7d36df45</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Alexander Wright</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>CHIEF EXECUTIVE OFFICER</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Nova Dynamics Inc.</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>+1 (415) 890-2341</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>alex@novadynamics.io</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>www.novadynamics.io</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>500 Howard St, Suite 400, San Francisco, CA 94105</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr"/>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="I13" s="13" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:37:37</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="K13" s="13" t="inlineStr">
         <is>
           <t>N
 Nova Dynamics Inc.
@@ -1207,42 +1269,42 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="120" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>f9a25cf5</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Gajan Gold</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Ganjan Gold</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>98792 40585</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr"/>
-      <c r="G13" s="10" t="inlineStr"/>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve"> A/G/12-A, Sardar Park-2, Opp. Swaminarayan School, GIDC, Ankleshwar-02.</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr"/>
-      <c r="J13" s="13" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:36:55</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>M Shree Gaajan Matay Namah I
 Ranchhodbhal
@@ -1257,42 +1319,42 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="120" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>4b26659b</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Kamlesh P. Soni</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Radhe Gold</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>+91 99130 67670, +91 99795 01319</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr"/>
+      <c r="G15" s="10" t="inlineStr"/>
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>9, Kuber Plaza Shopping Center,Tin Rasta Circle, Station Road.Ankleshwar-393 001</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="I15" s="13" t="inlineStr"/>
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:36:42</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K15" s="13" t="inlineStr">
         <is>
           <t>+91 99130 67670
 Ritesh P. Soni
@@ -1307,50 +1369,50 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>daa42bb7</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Arpana Shah</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr"/>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Shree paras jewellers </t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>98981 86861</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>sanjay_1964@yahoo.co.in</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr"/>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Ground Floor, "Tolani House" Station Road, Near Meghna Petrol Pump, Ankleshwar - 393 001</t>
         </is>
       </c>
-      <c r="I15" s="12" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>Paras Shah</t>
         </is>
       </c>
-      <c r="J15" s="13" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:35:35</t>
         </is>
       </c>
-      <c r="K15" s="12" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>Sanjay Shah
 Arpana Shah
@@ -1360,50 +1422,50 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="120" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>315ed1f9</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Nr. Swarnim Lakeview Park</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>NILESH SONI (Owner)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>PADMANABH GOLD</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>+91 99040 67969, +91 87808 30869</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>padmanabhgol6916@gmail.com</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>06, maruti Complex, Hansot Road, Anideshwar</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr"/>
-      <c r="J16" s="8" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr"/>
+      <c r="J17" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:35:01</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="K17" s="13" t="inlineStr">
         <is>
           <t>NILESH SONI (Owner)
 +91 99040 67969
@@ -1416,46 +1478,46 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="120" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>d08ea762</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Govindbhal Sonl</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr"/>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Ranuja Jewellers</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>8866808332, 8320454258</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr"/>
-      <c r="G17" s="10" t="inlineStr"/>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Chauta Bazar, Opp. Police Station, Ankleshwar - 39</t>
         </is>
       </c>
-      <c r="I17" s="12" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>Ranuja | DIAMOND / GOLD / SILVER</t>
         </is>
       </c>
-      <c r="J17" s="13" t="inlineStr">
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:33:28</t>
         </is>
       </c>
-      <c r="K17" s="12" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>Govindbhal Sonl
 Mo. : 8866808332
@@ -1467,46 +1529,46 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="108" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19" ht="108" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>b15cc6bd</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>un.r</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Suvarn mandir</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>+91 98250 99800, 9026741900, 4825094800</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>suwarn.mandir916@gamil.com</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr"/>
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>Nr. Markandeshwar Temple, Chauta Bazar, Ankleshwar (Guj.).</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr"/>
-      <c r="J18" s="8" t="inlineStr">
+      <c r="I19" s="13" t="inlineStr"/>
+      <c r="J19" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:32:24</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
+      <c r="K19" s="13" t="inlineStr">
         <is>
           <t>un.r
 Prinet Sari 9026741900
@@ -1517,46 +1579,46 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="120" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>2e7a3d64</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>ASHESHKUMAR BABULAL</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr"/>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>PADRAWALA    JEWELLERS</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>02642 260374, 98984 22541, 87330 38841</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr"/>
-      <c r="G19" s="10" t="inlineStr"/>
-      <c r="H19" s="12" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>KUBER PLAZA, TREN RA, Indraprasth Complex, Zadeshwar Road, BHARUCH.</t>
         </is>
       </c>
-      <c r="I19" s="12" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>S S JEWELLEN | GOLD • SILVER • DIAM | ANKLESHWAR-3931 | UTSAV | GOLD JEWELLERY | BIS HALLMARK | CHOKSHI | LAGADI / ORNAMENTS | GOLD &amp; SILVER COIN</t>
         </is>
       </c>
-      <c r="J19" s="13" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:29:26</t>
         </is>
       </c>
-      <c r="K19" s="12" t="inlineStr">
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>S S JEWELLEN
 GOLD • SILVER • DIAM
@@ -1580,38 +1642,38 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="72" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21" ht="72" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>fd368b98</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr"/>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Utsav jewellers </t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>94298 49555, 94271 75975</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr"/>
+      <c r="G21" s="10" t="inlineStr"/>
+      <c r="H21" s="13" t="inlineStr">
         <is>
           <t>Shop No.2-3-4, Kaji Shopping Center, Opp.Bank of Baroda, Station Road, Ankleshwar-393 001 Dist. Bharuch</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr"/>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="I21" s="13" t="inlineStr"/>
+      <c r="J21" s="14" t="inlineStr">
         <is>
           <t>2026-10-22 18:28:39</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
+      <c r="K21" s="13" t="inlineStr">
         <is>
           <t>Shop No.2-3-4, Kaji Shopping Center,
 Opp.Bank of Baroda, Station Road,
@@ -1620,31 +1682,10 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>b13e5aae</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr"/>
-      <c r="C21" s="10" t="inlineStr"/>
-      <c r="D21" s="10" t="inlineStr"/>
-      <c r="E21" s="11" t="inlineStr"/>
-      <c r="F21" s="10" t="inlineStr"/>
-      <c r="G21" s="10" t="inlineStr"/>
-      <c r="H21" s="12" t="inlineStr"/>
-      <c r="I21" s="12" t="inlineStr"/>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-22 18:28:28</t>
-        </is>
-      </c>
-      <c r="K21" s="12" t="inlineStr"/>
-    </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>986d6302</t>
+          <t>b13e5aae</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr"/>
@@ -1657,51 +1698,72 @@
       <c r="I22" s="7" t="inlineStr"/>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-22 18:28:23</t>
+          <t>2026-10-22 18:28:28</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr"/>
     </row>
-    <row r="23" ht="120" customHeight="1">
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>07bbfed8</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>GOLD • SILVER • DIAMOND</t>
-        </is>
-      </c>
+          <t>986d6302</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr"/>
       <c r="C23" s="10" t="inlineStr"/>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>SS JEWELLERS</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>7016622431, 7862822743</t>
-        </is>
-      </c>
+      <c r="D23" s="10" t="inlineStr"/>
+      <c r="E23" s="11" t="inlineStr"/>
       <c r="F23" s="10" t="inlineStr"/>
       <c r="G23" s="10" t="inlineStr"/>
-      <c r="H23" s="12" t="inlineStr">
+      <c r="H23" s="13" t="inlineStr"/>
+      <c r="I23" s="13" t="inlineStr"/>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:28:23</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr"/>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>07bbfed8</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>GOLD • SILVER • DIAMOND</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>SS JEWELLERS</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>7016622431, 7862822743</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>G-5. KUBER PLAZA, TEEN RASTA CIRCLE, ANKLESHWAR-393001.</t>
         </is>
       </c>
-      <c r="I23" s="12" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>SUNIL SONI | SAGAR SONI</t>
         </is>
       </c>
-      <c r="J23" s="13" t="inlineStr">
+      <c r="J24" s="8" t="inlineStr">
         <is>
           <t>2026-10-22 18:27:30</t>
         </is>
       </c>
-      <c r="K23" s="12" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>SUNIL SONI
 SAGAR SONI
@@ -1714,42 +1776,42 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>4712d499</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>SHAILESH SONI</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr"/>
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">RADHE KRISHNA JEWELLERS </t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>9327962757</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr"/>
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve"> Shop No.3, Patel Vitthal Co-Op Society, Nr. Shital Circle, Kasak, Bharuch.</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr"/>
-      <c r="J24" s="8" t="inlineStr">
+      <c r="I25" s="13" t="inlineStr"/>
+      <c r="J25" s="14" t="inlineStr">
         <is>
           <t>2026-10-21 18:08:55</t>
         </is>
       </c>
-      <c r="K24" s="7" t="inlineStr">
+      <c r="K25" s="13" t="inlineStr">
         <is>
           <t>제어라: 자외되려가격요
 Specialist in all types of gold and silver
@@ -1759,38 +1821,38 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="120" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>7ea80899</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr"/>
-      <c r="C25" s="10" t="inlineStr"/>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>MITTAL  JEWELLERS</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>9825505477</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr"/>
-      <c r="G25" s="10" t="inlineStr"/>
-      <c r="H25" s="12" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>218, ORION ARCADE, Zadeshwar Road, Bharuch</t>
         </is>
       </c>
-      <c r="I25" s="12" t="inlineStr"/>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr"/>
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>2026-10-21 18:04:14</t>
         </is>
       </c>
-      <c r="K25" s="12" t="inlineStr">
+      <c r="K26" s="7" t="inlineStr">
         <is>
           <t>영리 에리리
 Mo. : 9825505477
@@ -1802,38 +1864,38 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="120" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>c739c03a</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>O GIHIS - CIN- DINOTECA</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr"/>
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>RouPS</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr"/>
-      <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="7" t="inlineStr"/>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr"/>
+      <c r="F27" s="10" t="inlineStr"/>
+      <c r="G27" s="10" t="inlineStr"/>
+      <c r="H27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>@ CSi E21 . 211421 | 03521E- 2410iE | 5.0 | Fisim. | 2 | visit Dell d | ตาหมาล -(มหยก | 3 2isdpcz-미국리. | 29- | 30 | 1 - 12- | 12 | 11 - | 2026 | 2026 | 2026 | 27. | /1 - | 2026 | 2026 | 2026 | Days： | eryx | SailE | ตาคงเล - หรอยมก | 25-18-2026 | - 6/12/2026 | 2 kux | 122122 | aia zusaiz zusaia. | ม. CoCO R2222 | ) | kip | | | Rett | ٧٤٩ ٠ | 8 Paga</t>
         </is>
       </c>
-      <c r="J26" s="8" t="inlineStr">
+      <c r="J27" s="14" t="inlineStr">
         <is>
           <t>2026-10-21 17:57:18</t>
         </is>
       </c>
-      <c r="K26" s="7" t="inlineStr">
+      <c r="K27" s="13" t="inlineStr">
         <is>
           <t>RouPS
 @ CSi E21 . 211421
@@ -1878,42 +1940,42 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="120" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="28" ht="120" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>5412ebae</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>HIMANSHU</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr"/>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">DHANLAXMI JEWELLERS </t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve"> 76007 68851</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr"/>
-      <c r="G27" s="10" t="inlineStr"/>
-      <c r="H27" s="12" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">7/8, Mahajan Market, Sevashram Road, Panchbatti, BHARUCH </t>
         </is>
       </c>
-      <c r="I27" s="12" t="inlineStr"/>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="I28" s="7" t="inlineStr"/>
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>2026-10-21 17:56:19</t>
         </is>
       </c>
-      <c r="K27" s="12" t="inlineStr">
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>DHRUV
 DEVENDRA SONI
@@ -1928,42 +1990,42 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="120" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="29" ht="120" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>a12c2b06</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>J. K. JEWELLERS</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>02642 - 241576, 98241 27077</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr"/>
-      <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="F29" s="10" t="inlineStr"/>
+      <c r="G29" s="10" t="inlineStr"/>
+      <c r="H29" s="13" t="inlineStr">
         <is>
           <t>Near Rungta School, Station Road, Bharuch-392 001.</t>
         </is>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I29" s="13" t="inlineStr">
         <is>
           <t>GOVT APPROVED VALUER | YOUR TRUST SINCE 100 YEARS | Exclusive Gold, Silver &amp; Diamond Jewellery | WE DO NOT HAVE ANY BRANCH</t>
         </is>
       </c>
-      <c r="J28" s="8" t="inlineStr">
+      <c r="J29" s="14" t="inlineStr">
         <is>
           <t>2026-10-21 17:49:41</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr">
+      <c r="K29" s="13" t="inlineStr">
         <is>
           <t>GOVT APPROVED VALUER
 Ph. : 02642 - 241576
@@ -1976,46 +2038,46 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="120" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="30" ht="120" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>654a39c4</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>BHAGWANDAS</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr"/>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>JEWELLERS</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>98254 22209, 78745 85140</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr"/>
-      <c r="G29" s="10" t="inlineStr"/>
-      <c r="H29" s="12" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>1, Daudi Shopping Center, Panchbatti, Bharuch 392 001</t>
         </is>
       </c>
-      <c r="I29" s="12" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>Since 1933 | Gold &amp; Silver Merchant</t>
         </is>
       </c>
-      <c r="J29" s="13" t="inlineStr">
+      <c r="J30" s="8" t="inlineStr">
         <is>
           <t>2026-10-21 17:48:11</t>
         </is>
       </c>
-      <c r="K29" s="12" t="inlineStr">
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>Since 1933
 BHAGWANDAS
@@ -2027,46 +2089,46 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="120" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="31" ht="120" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>91bca1e7</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>SONI BROTHERS</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr"/>
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>SB</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>99241 12662, 98981 09155</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr"/>
-      <c r="G30" s="4" t="inlineStr"/>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr"/>
+      <c r="G31" s="10" t="inlineStr"/>
+      <c r="H31" s="13" t="inlineStr">
         <is>
           <t>(02642) 268290, Bharuch - 392001</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
+      <c r="I31" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Navadera, Nr. Datt Temple, BHARUCH </t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
+      <c r="J31" s="14" t="inlineStr">
         <is>
           <t>2026-10-21 17:46:12</t>
         </is>
       </c>
-      <c r="K30" s="7" t="inlineStr">
+      <c r="K31" s="13" t="inlineStr">
         <is>
           <t>(02642) 268290
 Bakulbhai: 99241 12662
@@ -2079,50 +2141,50 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="120" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="32" ht="120" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>693bd944</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>BARDOLI •</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr"/>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr"/>
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Mahendra jew</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>98795 46186, 82387 65476</t>
         </is>
       </c>
-      <c r="F31" s="14" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>mahendrajewellers2006@gmail.com</t>
         </is>
       </c>
-      <c r="G31" s="10" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>Station Road, Bardoli.</t>
         </is>
       </c>
-      <c r="I31" s="12" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>• MADHI • | Pin : 394 601 | A/2, Sardar Arcade, | Main Bazar, Madhi. Pin : 394 340</t>
         </is>
       </c>
-      <c r="J31" s="13" t="inlineStr">
+      <c r="J32" s="8" t="inlineStr">
         <is>
           <t>2026-10-21 17:46:11</t>
         </is>
       </c>
-      <c r="K31" s="12" t="inlineStr">
+      <c r="K32" s="7" t="inlineStr">
         <is>
           <t>2시8회 어제르의
 • MADHI •
@@ -2137,71 +2199,71 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>7f98ce42</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr"/>
-      <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr"/>
-      <c r="H32" s="7" t="inlineStr"/>
-      <c r="I32" s="7" t="inlineStr"/>
-      <c r="J32" s="8" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr"/>
+      <c r="C33" s="10" t="inlineStr"/>
+      <c r="D33" s="10" t="inlineStr"/>
+      <c r="E33" s="11" t="inlineStr"/>
+      <c r="F33" s="10" t="inlineStr"/>
+      <c r="G33" s="10" t="inlineStr"/>
+      <c r="H33" s="13" t="inlineStr"/>
+      <c r="I33" s="13" t="inlineStr"/>
+      <c r="J33" s="14" t="inlineStr">
         <is>
           <t>2026-10-21 17:45:51</t>
         </is>
       </c>
-      <c r="K32" s="7" t="inlineStr"/>
-    </row>
-    <row r="33" ht="120" customHeight="1">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="K33" s="13" t="inlineStr"/>
+    </row>
+    <row r="34" ht="120" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>dbb845b1</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">KESHAR JEWELLERS </t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr"/>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>SIP.N</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>98240 31510, 99982 68342</t>
         </is>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>kesharjewellers@yahoo.com</t>
         </is>
       </c>
-      <c r="G33" s="10" t="inlineStr"/>
-      <c r="H33" s="12" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>SB-16, Shri Niketan Resi Plaza, Nr. Jyoti Nagar, Zadeshwar Road, Bharuch.</t>
         </is>
       </c>
-      <c r="I33" s="12" t="inlineStr">
+      <c r="I34" s="7" t="inlineStr">
         <is>
           <t>Deval Dodiya</t>
         </is>
       </c>
-      <c r="J33" s="13" t="inlineStr">
+      <c r="J34" s="8" t="inlineStr">
         <is>
           <t>2026-10-21 17:42:11</t>
         </is>
       </c>
-      <c r="K33" s="12" t="inlineStr">
+      <c r="K34" s="7" t="inlineStr">
         <is>
           <t>SIP.N
 98240 31510
@@ -2214,44 +2276,46 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>43876b56</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="5" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr"/>
-      <c r="H34" s="7" t="inlineStr"/>
-      <c r="I34" s="7" t="inlineStr"/>
-      <c r="J34" s="8" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr"/>
+      <c r="C35" s="10" t="inlineStr"/>
+      <c r="D35" s="10" t="inlineStr"/>
+      <c r="E35" s="11" t="inlineStr"/>
+      <c r="F35" s="10" t="inlineStr"/>
+      <c r="G35" s="10" t="inlineStr"/>
+      <c r="H35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr"/>
+      <c r="J35" s="14" t="inlineStr">
         <is>
           <t>2026-10-21 17:41:52</t>
         </is>
       </c>
-      <c r="K34" s="7" t="inlineStr"/>
+      <c r="K35" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K34"/>
+  <autoFilter ref="A1:K35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>